<commit_message>
one workbook and one figure PDF per step, same numbers, fewer files
</commit_message>
<xml_diff>
--- a/01_Preprocess/03_Imputation/c_data/03_impute.xlsx
+++ b/01_Preprocess/03_Imputation/c_data/03_impute.xlsx
@@ -7,14 +7,41 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="imputation" sheetId="1" r:id="rId1"/>
+    <sheet name="read_me" sheetId="1" r:id="rId1"/>
+    <sheet name="imputation" sheetId="2" r:id="rId2"/>
+    <sheet name="input_manifest" sheetId="3" r:id="rId3"/>
+    <sheet name="package_versions" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="110">
+  <si>
+    <t>sheet</t>
+  </si>
+  <si>
+    <t>holds</t>
+  </si>
+  <si>
+    <t>imputation</t>
+  </si>
+  <si>
+    <t>missForest settings, share of values imputed, out-of-bag error.</t>
+  </si>
+  <si>
+    <t>input_manifest</t>
+  </si>
+  <si>
+    <t>Files read, with md5.</t>
+  </si>
+  <si>
+    <t>package_versions</t>
+  </si>
+  <si>
+    <t>Packages loaded at run time.</t>
+  </si>
   <si>
     <t>method</t>
   </si>
@@ -38,6 +65,288 @@
   </si>
   <si>
     <t>ranger</t>
+  </si>
+  <si>
+    <t>input</t>
+  </si>
+  <si>
+    <t>path</t>
+  </si>
+  <si>
+    <t>md5</t>
+  </si>
+  <si>
+    <t>normalized</t>
+  </si>
+  <si>
+    <t>01_Preprocess/02_Normalization/c_data/DAList_normalized.rds</t>
+  </si>
+  <si>
+    <t>01097241ebec0987911c1232265b9377</t>
+  </si>
+  <si>
+    <t>package</t>
+  </si>
+  <si>
+    <t>version</t>
+  </si>
+  <si>
+    <t>source</t>
+  </si>
+  <si>
+    <t>BiocManager</t>
+  </si>
+  <si>
+    <t>1.30.27</t>
+  </si>
+  <si>
+    <t>CRAN (R 4.6.0)</t>
+  </si>
+  <si>
+    <t>cli</t>
+  </si>
+  <si>
+    <t>3.6.6</t>
+  </si>
+  <si>
+    <t>codetools</t>
+  </si>
+  <si>
+    <t>0.2-20</t>
+  </si>
+  <si>
+    <t>digest</t>
+  </si>
+  <si>
+    <t>0.6.39</t>
+  </si>
+  <si>
+    <t>doRNG</t>
+  </si>
+  <si>
+    <t>1.8.6.3</t>
+  </si>
+  <si>
+    <t>dplyr</t>
+  </si>
+  <si>
+    <t>1.2.1</t>
+  </si>
+  <si>
+    <t>evaluate</t>
+  </si>
+  <si>
+    <t>1.0.5</t>
+  </si>
+  <si>
+    <t>fastmap</t>
+  </si>
+  <si>
+    <t>1.2.0</t>
+  </si>
+  <si>
+    <t>foreach</t>
+  </si>
+  <si>
+    <t>1.5.2</t>
+  </si>
+  <si>
+    <t>generics</t>
+  </si>
+  <si>
+    <t>0.1.4</t>
+  </si>
+  <si>
+    <t>glue</t>
+  </si>
+  <si>
+    <t>1.8.1</t>
+  </si>
+  <si>
+    <t>here</t>
+  </si>
+  <si>
+    <t>1.0.2</t>
+  </si>
+  <si>
+    <t>htmltools</t>
+  </si>
+  <si>
+    <t>0.5.9</t>
+  </si>
+  <si>
+    <t>htmlwidgets</t>
+  </si>
+  <si>
+    <t>1.6.4</t>
+  </si>
+  <si>
+    <t>iterators</t>
+  </si>
+  <si>
+    <t>1.0.14</t>
+  </si>
+  <si>
+    <t>itertools</t>
+  </si>
+  <si>
+    <t>0.1-3</t>
+  </si>
+  <si>
+    <t>jsonlite</t>
+  </si>
+  <si>
+    <t>2.0.0</t>
+  </si>
+  <si>
+    <t>knitr</t>
+  </si>
+  <si>
+    <t>1.51</t>
+  </si>
+  <si>
+    <t>lattice</t>
+  </si>
+  <si>
+    <t>0.22-9</t>
+  </si>
+  <si>
+    <t>lifecycle</t>
+  </si>
+  <si>
+    <t>magrittr</t>
+  </si>
+  <si>
+    <t>2.0.5</t>
+  </si>
+  <si>
+    <t>Matrix</t>
+  </si>
+  <si>
+    <t>1.7-5</t>
+  </si>
+  <si>
+    <t>1.6.1</t>
+  </si>
+  <si>
+    <t>otel</t>
+  </si>
+  <si>
+    <t>0.2.0</t>
+  </si>
+  <si>
+    <t>pillar</t>
+  </si>
+  <si>
+    <t>1.11.1</t>
+  </si>
+  <si>
+    <t>pkgconfig</t>
+  </si>
+  <si>
+    <t>2.0.3</t>
+  </si>
+  <si>
+    <t>R6</t>
+  </si>
+  <si>
+    <t>2.6.1</t>
+  </si>
+  <si>
+    <t>randomForest</t>
+  </si>
+  <si>
+    <t>4.7-1.2</t>
+  </si>
+  <si>
+    <t>0.18.0</t>
+  </si>
+  <si>
+    <t>rbibutils</t>
+  </si>
+  <si>
+    <t>2.4.1</t>
+  </si>
+  <si>
+    <t>Rcpp</t>
+  </si>
+  <si>
+    <t>1.1.1-1.1</t>
+  </si>
+  <si>
+    <t>Rdpack</t>
+  </si>
+  <si>
+    <t>2.6.6</t>
+  </si>
+  <si>
+    <t>renv</t>
+  </si>
+  <si>
+    <t>1.2.3</t>
+  </si>
+  <si>
+    <t>rlang</t>
+  </si>
+  <si>
+    <t>1.3.0</t>
+  </si>
+  <si>
+    <t>CRAN (R 4.6.1)</t>
+  </si>
+  <si>
+    <t>rmarkdown</t>
+  </si>
+  <si>
+    <t>2.31</t>
+  </si>
+  <si>
+    <t>rngtools</t>
+  </si>
+  <si>
+    <t>rprojroot</t>
+  </si>
+  <si>
+    <t>2.1.1</t>
+  </si>
+  <si>
+    <t>sessioninfo</t>
+  </si>
+  <si>
+    <t>1.2.4</t>
+  </si>
+  <si>
+    <t>tibble</t>
+  </si>
+  <si>
+    <t>3.3.1</t>
+  </si>
+  <si>
+    <t>tidyselect</t>
+  </si>
+  <si>
+    <t>vctrs</t>
+  </si>
+  <si>
+    <t>0.7.3</t>
+  </si>
+  <si>
+    <t>writexl</t>
+  </si>
+  <si>
+    <t>2.0.1</t>
+  </si>
+  <si>
+    <t>xfun</t>
+  </si>
+  <si>
+    <t>0.57</t>
+  </si>
+  <si>
+    <t>yaml</t>
+  </si>
+  <si>
+    <t>2.3.12</t>
   </si>
 </sst>
 </file>
@@ -380,35 +689,77 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C2">
         <v>10</v>
@@ -421,6 +772,543 @@
       </c>
       <c r="F2">
         <v>0.1514637503795072</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B15" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" t="s">
+        <v>57</v>
+      </c>
+      <c r="C17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>58</v>
+      </c>
+      <c r="B18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" t="s">
+        <v>62</v>
+      </c>
+      <c r="B20" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" t="s">
+        <v>64</v>
+      </c>
+      <c r="B21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" t="s">
+        <v>65</v>
+      </c>
+      <c r="B22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C22" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" t="s">
+        <v>67</v>
+      </c>
+      <c r="B23" t="s">
+        <v>68</v>
+      </c>
+      <c r="C23" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" t="s">
+        <v>14</v>
+      </c>
+      <c r="B24" t="s">
+        <v>69</v>
+      </c>
+      <c r="C24" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
+        <v>70</v>
+      </c>
+      <c r="B25" t="s">
+        <v>71</v>
+      </c>
+      <c r="C25" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" t="s">
+        <v>72</v>
+      </c>
+      <c r="B26" t="s">
+        <v>73</v>
+      </c>
+      <c r="C26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" t="s">
+        <v>74</v>
+      </c>
+      <c r="B27" t="s">
+        <v>75</v>
+      </c>
+      <c r="C27" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" t="s">
+        <v>76</v>
+      </c>
+      <c r="B28" t="s">
+        <v>77</v>
+      </c>
+      <c r="C28" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" t="s">
+        <v>78</v>
+      </c>
+      <c r="B29" t="s">
+        <v>79</v>
+      </c>
+      <c r="C29" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" t="s">
+        <v>15</v>
+      </c>
+      <c r="B30" t="s">
+        <v>80</v>
+      </c>
+      <c r="C30" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
+        <v>81</v>
+      </c>
+      <c r="B31" t="s">
+        <v>82</v>
+      </c>
+      <c r="C31" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
+        <v>83</v>
+      </c>
+      <c r="B32" t="s">
+        <v>84</v>
+      </c>
+      <c r="C32" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" t="s">
+        <v>85</v>
+      </c>
+      <c r="B33" t="s">
+        <v>86</v>
+      </c>
+      <c r="C33" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" t="s">
+        <v>87</v>
+      </c>
+      <c r="B34" t="s">
+        <v>88</v>
+      </c>
+      <c r="C34" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" t="s">
+        <v>89</v>
+      </c>
+      <c r="B35" t="s">
+        <v>90</v>
+      </c>
+      <c r="C35" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" t="s">
+        <v>92</v>
+      </c>
+      <c r="B36" t="s">
+        <v>93</v>
+      </c>
+      <c r="C36" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" t="s">
+        <v>94</v>
+      </c>
+      <c r="B37" t="s">
+        <v>43</v>
+      </c>
+      <c r="C37" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
+        <v>95</v>
+      </c>
+      <c r="B38" t="s">
+        <v>96</v>
+      </c>
+      <c r="C38" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
+        <v>97</v>
+      </c>
+      <c r="B39" t="s">
+        <v>98</v>
+      </c>
+      <c r="C39" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
+        <v>99</v>
+      </c>
+      <c r="B40" t="s">
+        <v>100</v>
+      </c>
+      <c r="C40" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
+        <v>101</v>
+      </c>
+      <c r="B41" t="s">
+        <v>37</v>
+      </c>
+      <c r="C41" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" t="s">
+        <v>102</v>
+      </c>
+      <c r="B42" t="s">
+        <v>103</v>
+      </c>
+      <c r="C42" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" t="s">
+        <v>104</v>
+      </c>
+      <c r="B43" t="s">
+        <v>105</v>
+      </c>
+      <c r="C43" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" t="s">
+        <v>106</v>
+      </c>
+      <c r="B44" t="s">
+        <v>107</v>
+      </c>
+      <c r="C44" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" t="s">
+        <v>108</v>
+      </c>
+      <c r="B45" t="s">
+        <v>109</v>
+      </c>
+      <c r="C45" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
inputs become plain data and preprocessing becomes plain R, same DALists to the byte
</commit_message>
<xml_diff>
--- a/01_Preprocess/03_Imputation/c_data/03_impute.xlsx
+++ b/01_Preprocess/03_Imputation/c_data/03_impute.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="93">
   <si>
     <t>sheet</t>
   </si>
@@ -133,87 +133,54 @@
     <t>1.2.1</t>
   </si>
   <si>
-    <t>evaluate</t>
+    <t>foreach</t>
+  </si>
+  <si>
+    <t>1.5.2</t>
+  </si>
+  <si>
+    <t>generics</t>
+  </si>
+  <si>
+    <t>0.1.4</t>
+  </si>
+  <si>
+    <t>glue</t>
+  </si>
+  <si>
+    <t>1.8.1</t>
+  </si>
+  <si>
+    <t>here</t>
+  </si>
+  <si>
+    <t>1.0.2</t>
+  </si>
+  <si>
+    <t>iterators</t>
+  </si>
+  <si>
+    <t>1.0.14</t>
+  </si>
+  <si>
+    <t>itertools</t>
+  </si>
+  <si>
+    <t>0.1-3</t>
+  </si>
+  <si>
+    <t>lattice</t>
+  </si>
+  <si>
+    <t>0.22-9</t>
+  </si>
+  <si>
+    <t>lifecycle</t>
   </si>
   <si>
     <t>1.0.5</t>
   </si>
   <si>
-    <t>fastmap</t>
-  </si>
-  <si>
-    <t>1.2.0</t>
-  </si>
-  <si>
-    <t>foreach</t>
-  </si>
-  <si>
-    <t>1.5.2</t>
-  </si>
-  <si>
-    <t>generics</t>
-  </si>
-  <si>
-    <t>0.1.4</t>
-  </si>
-  <si>
-    <t>glue</t>
-  </si>
-  <si>
-    <t>1.8.1</t>
-  </si>
-  <si>
-    <t>here</t>
-  </si>
-  <si>
-    <t>1.0.2</t>
-  </si>
-  <si>
-    <t>htmltools</t>
-  </si>
-  <si>
-    <t>0.5.9</t>
-  </si>
-  <si>
-    <t>htmlwidgets</t>
-  </si>
-  <si>
-    <t>1.6.4</t>
-  </si>
-  <si>
-    <t>iterators</t>
-  </si>
-  <si>
-    <t>1.0.14</t>
-  </si>
-  <si>
-    <t>itertools</t>
-  </si>
-  <si>
-    <t>0.1-3</t>
-  </si>
-  <si>
-    <t>jsonlite</t>
-  </si>
-  <si>
-    <t>2.0.0</t>
-  </si>
-  <si>
-    <t>knitr</t>
-  </si>
-  <si>
-    <t>1.51</t>
-  </si>
-  <si>
-    <t>lattice</t>
-  </si>
-  <si>
-    <t>0.22-9</t>
-  </si>
-  <si>
-    <t>lifecycle</t>
-  </si>
-  <si>
     <t>magrittr</t>
   </si>
   <si>
@@ -229,12 +196,6 @@
     <t>1.6.1</t>
   </si>
   <si>
-    <t>otel</t>
-  </si>
-  <si>
-    <t>0.2.0</t>
-  </si>
-  <si>
     <t>pillar</t>
   </si>
   <si>
@@ -295,12 +256,6 @@
     <t>CRAN (R 4.6.1)</t>
   </si>
   <si>
-    <t>rmarkdown</t>
-  </si>
-  <si>
-    <t>2.31</t>
-  </si>
-  <si>
     <t>rngtools</t>
   </si>
   <si>
@@ -335,12 +290,6 @@
   </si>
   <si>
     <t>2.0.1</t>
-  </si>
-  <si>
-    <t>xfun</t>
-  </si>
-  <si>
-    <t>0.57</t>
   </si>
   <si>
     <t>yaml</t>
@@ -813,7 +762,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -1005,10 +954,10 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" t="s">
         <v>58</v>
-      </c>
-      <c r="B18" t="s">
-        <v>59</v>
       </c>
       <c r="C18" t="s">
         <v>27</v>
@@ -1016,10 +965,10 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
+        <v>59</v>
+      </c>
+      <c r="B19" t="s">
         <v>60</v>
-      </c>
-      <c r="B19" t="s">
-        <v>61</v>
       </c>
       <c r="C19" t="s">
         <v>27</v>
@@ -1027,10 +976,10 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" t="s">
         <v>62</v>
-      </c>
-      <c r="B20" t="s">
-        <v>63</v>
       </c>
       <c r="C20" t="s">
         <v>27</v>
@@ -1038,10 +987,10 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
+        <v>63</v>
+      </c>
+      <c r="B21" t="s">
         <v>64</v>
-      </c>
-      <c r="B21" t="s">
-        <v>39</v>
       </c>
       <c r="C21" t="s">
         <v>27</v>
@@ -1060,10 +1009,10 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
+        <v>15</v>
+      </c>
+      <c r="B23" t="s">
         <v>67</v>
-      </c>
-      <c r="B23" t="s">
-        <v>68</v>
       </c>
       <c r="C23" t="s">
         <v>27</v>
@@ -1071,7 +1020,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>14</v>
+        <v>68</v>
       </c>
       <c r="B24" t="s">
         <v>69</v>
@@ -1121,15 +1070,15 @@
         <v>77</v>
       </c>
       <c r="C28" t="s">
-        <v>27</v>
+        <v>78</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B29" t="s">
-        <v>79</v>
+        <v>39</v>
       </c>
       <c r="C29" t="s">
         <v>27</v>
@@ -1137,10 +1086,10 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>15</v>
+        <v>80</v>
       </c>
       <c r="B30" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C30" t="s">
         <v>27</v>
@@ -1148,10 +1097,10 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B31" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C31" t="s">
         <v>27</v>
@@ -1159,10 +1108,10 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B32" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C32" t="s">
         <v>27</v>
@@ -1170,10 +1119,10 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B33" t="s">
-        <v>86</v>
+        <v>37</v>
       </c>
       <c r="C33" t="s">
         <v>27</v>
@@ -1198,116 +1147,17 @@
         <v>90</v>
       </c>
       <c r="C35" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
+        <v>91</v>
+      </c>
+      <c r="B36" t="s">
         <v>92</v>
       </c>
-      <c r="B36" t="s">
-        <v>93</v>
-      </c>
       <c r="C36" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3">
-      <c r="A37" t="s">
-        <v>94</v>
-      </c>
-      <c r="B37" t="s">
-        <v>43</v>
-      </c>
-      <c r="C37" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3">
-      <c r="A38" t="s">
-        <v>95</v>
-      </c>
-      <c r="B38" t="s">
-        <v>96</v>
-      </c>
-      <c r="C38" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3">
-      <c r="A39" t="s">
-        <v>97</v>
-      </c>
-      <c r="B39" t="s">
-        <v>98</v>
-      </c>
-      <c r="C39" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3">
-      <c r="A40" t="s">
-        <v>99</v>
-      </c>
-      <c r="B40" t="s">
-        <v>100</v>
-      </c>
-      <c r="C40" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3">
-      <c r="A41" t="s">
-        <v>101</v>
-      </c>
-      <c r="B41" t="s">
-        <v>37</v>
-      </c>
-      <c r="C41" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3">
-      <c r="A42" t="s">
-        <v>102</v>
-      </c>
-      <c r="B42" t="s">
-        <v>103</v>
-      </c>
-      <c r="C42" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3">
-      <c r="A43" t="s">
-        <v>104</v>
-      </c>
-      <c r="B43" t="s">
-        <v>105</v>
-      </c>
-      <c r="C43" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3">
-      <c r="A44" t="s">
-        <v>106</v>
-      </c>
-      <c r="B44" t="s">
-        <v>107</v>
-      </c>
-      <c r="C44" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3">
-      <c r="A45" t="s">
-        <v>108</v>
-      </c>
-      <c r="B45" t="s">
-        <v>109</v>
-      </c>
-      <c r="C45" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
rerun everything end to end; old numbers hold, new ones only where we asked
</commit_message>
<xml_diff>
--- a/01_Preprocess/03_Imputation/c_data/03_impute.xlsx
+++ b/01_Preprocess/03_Imputation/c_data/03_impute.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="91">
   <si>
     <t>sheet</t>
   </si>
@@ -290,12 +290,6 @@
   </si>
   <si>
     <t>2.0.1</t>
-  </si>
-  <si>
-    <t>yaml</t>
-  </si>
-  <si>
-    <t>2.3.12</t>
   </si>
 </sst>
 </file>
@@ -762,7 +756,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -1150,17 +1144,6 @@
         <v>78</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
-      <c r="A36" t="s">
-        <v>91</v>
-      </c>
-      <c r="B36" t="s">
-        <v>92</v>
-      </c>
-      <c r="C36" t="s">
-        <v>27</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
rerun all twenty-one steps on the new scripts; modules now number fifteen
</commit_message>
<xml_diff>
--- a/01_Preprocess/03_Imputation/c_data/03_impute.xlsx
+++ b/01_Preprocess/03_Imputation/c_data/03_impute.xlsx
@@ -82,7 +82,7 @@
     <t>01_Preprocess/02_Normalization/c_data/DAList_normalized.rds</t>
   </si>
   <si>
-    <t>01097241ebec0987911c1232265b9377</t>
+    <t>3759b18a8f3aa42799daa3bda21b03fa</t>
   </si>
   <si>
     <t>package</t>
@@ -714,7 +714,7 @@
         <v>12.26783625730994</v>
       </c>
       <c r="F2">
-        <v>0.1514637503795072</v>
+        <v>0.150501570976779</v>
       </c>
     </row>
   </sheetData>

</xml_diff>